<commit_message>
Akademik faoliyat (Adabiyotlar) bo'limi, modal oynasi va server konfiguratsiyalari qo'shildi
</commit_message>
<xml_diff>
--- a/file/sertifikat.xlsx
+++ b/file/sertifikat.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7C4283-8559-4171-8AD3-FFAF36062406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2D816B4-811A-4223-9401-775FFF14CC0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>№</t>
   </si>
@@ -51,21 +51,6 @@
   </si>
   <si>
     <t>Fakulteti</t>
-  </si>
-  <si>
-    <t>Aassa</t>
-  </si>
-  <si>
-    <t>ASAD</t>
-  </si>
-  <si>
-    <t>asssa</t>
-  </si>
-  <si>
-    <t>rt</t>
-  </si>
-  <si>
-    <t>tr</t>
   </si>
 </sst>
 </file>
@@ -451,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" customWidth="1"/>
@@ -462,7 +447,7 @@
     <col min="8" max="12" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,121 +484,73 @@
       <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
-      <c r="B2" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="B2" s="3"/>
       <c r="C2" s="4"/>
-      <c r="D2" s="3">
-        <v>234234</v>
-      </c>
-      <c r="E2" s="3">
-        <v>342</v>
-      </c>
-      <c r="F2" s="3">
-        <v>2342</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
     </row>
-    <row r="3" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="B3" s="3"/>
       <c r="C3" s="4"/>
-      <c r="D3" s="3">
-        <v>234234</v>
-      </c>
-      <c r="E3" s="3">
-        <v>234</v>
-      </c>
-      <c r="F3" s="3">
-        <v>342</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
     </row>
-    <row r="4" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="B4" s="3"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="3">
-        <v>234234</v>
-      </c>
-      <c r="E4" s="3">
-        <v>4</v>
-      </c>
-      <c r="F4" s="3">
-        <v>342</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
     </row>
-    <row r="5" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
-      <c r="B5" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="B5" s="3"/>
       <c r="C5" s="4"/>
-      <c r="D5" s="3">
-        <v>234234</v>
-      </c>
-      <c r="E5" s="3">
-        <v>34</v>
-      </c>
-      <c r="F5" s="3">
-        <v>342</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
     </row>
-    <row r="6" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="3" t="s">
-        <v>14</v>
-      </c>
+      <c r="B6" s="3"/>
       <c r="C6" s="4"/>
-      <c r="D6" s="3">
-        <v>234234</v>
-      </c>
-      <c r="E6" s="3">
-        <v>2342</v>
-      </c>
-      <c r="F6" s="3">
-        <v>34</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>

</xml_diff>